<commit_message>
Liga de Excel a OC
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/PROVEEDORES.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/PROVEEDORES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maria Luisa Martinez\Documents\NetBeansProjects\OCXRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DE0785-174D-4180-960D-591814A545B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" xr2:uid="{EBE529F0-1989-4E0B-B87D-8E5A162CA571}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EBE529F0-1989-4E0B-B87D-8E5A162CA571}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Terminos y condiciones del PDF
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/PROVEEDORES.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/PROVEEDORES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5138D754-9E59-4850-BD4B-9551CA94B37D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7F9B31-674D-422D-AF7F-3579EB7A68BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EBE529F0-1989-4E0B-B87D-8E5A162CA571}"/>
   </bookViews>
@@ -62,9 +62,6 @@
     <t>bimb26</t>
   </si>
   <si>
-    <t>BIMBO SA DE CV</t>
-  </si>
-  <si>
     <t>BMB230326XXRRFS</t>
   </si>
   <si>
@@ -99,6 +96,9 @@
   </si>
   <si>
     <t>PUE (Pago en una sola exhibición)</t>
+  </si>
+  <si>
+    <t>BIMBO S.A. DE C.V.</t>
   </si>
 </sst>
 </file>
@@ -514,22 +514,22 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
         <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -537,34 +537,34 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
       </c>
       <c r="D2">
         <v>5543647896</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>